<commit_message>
Publish browser tools and improve Excel report tables and task flow
</commit_message>
<xml_diff>
--- a/docs/peak-results-template.xlsx
+++ b/docs/peak-results-template.xlsx
@@ -2,8 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peak Results" sheetId="1" r:id="R4812c236fe91487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peak Results" sheetId="1" r:id="R51ac1bad11d84678"/>
   </x:sheets>
+  <x:definedNames>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Peak Results'!$A$2:$G$8</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="0">'Peak Results'!$6:$6</x:definedName>
+  </x:definedNames>
 </x:workbook>
 </file>
 
@@ -13,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0.00"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -45,7 +50,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -62,8 +67,23 @@
         <x:fgColor rgb="FFFFF8DF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF0F5FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D4ED8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border>
       <x:left/>
       <x:right/>
@@ -71,11 +91,26 @@
       <x:bottom/>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE2E8F0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE2E8F0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE2E8F0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE2E8F0"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -107,6 +142,84 @@
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -118,7 +231,6 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PeakResults" displayName="PeakResults" ref="A6:G8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:G8"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Band/Config"/>
     <x:tableColumn id="2" name="Channel"/>
@@ -327,19 +439,20 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
     <x:tabColor rgb="FF1D4ED8"/>
+    <x:pageSetUpPr fitToPage="1"/>
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="24" customHeight="1">
+    <x:row r="1" ht="10" customHeight="1">
       <x:c r="A1" s="1"/>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -348,102 +461,100 @@
       <x:c r="F1" s="1"/>
       <x:c r="G1" s="1"/>
     </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="2" t="str">
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="16" t="str">
         <x:v>Peak 測試結果</x:v>
       </x:c>
-      <x:c r="B2" s="1"/>
-      <x:c r="C2" s="1"/>
-      <x:c r="D2" s="1"/>
-      <x:c r="E2" s="1"/>
-      <x:c r="F2" s="1"/>
-      <x:c r="G2" s="1"/>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="3" t="str">
-        <x:v>SU / MU unit: Mbps. Gain is manually entered; no calculation.</x:v>
-      </x:c>
-      <x:c r="B3" s="1"/>
-      <x:c r="C3" s="1"/>
-      <x:c r="D3" s="1"/>
-      <x:c r="E3" s="1"/>
-      <x:c r="F3" s="1"/>
-      <x:c r="G3" s="1"/>
-    </x:row>
-    <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="3" t="str">
-        <x:v>Source: Empty template. No measured values supplied.</x:v>
-      </x:c>
-      <x:c r="B4" s="1"/>
-      <x:c r="C4" s="1"/>
-      <x:c r="D4" s="1"/>
-      <x:c r="E4" s="1"/>
-      <x:c r="F4" s="1"/>
-      <x:c r="G4" s="1"/>
-    </x:row>
-    <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="3" t="str">
-        <x:v>One row per Band/Config, Channel and Direction. Edit cells or use the table filter.</x:v>
-      </x:c>
-      <x:c r="B5" s="1"/>
-      <x:c r="C5" s="1"/>
-      <x:c r="D5" s="1"/>
-      <x:c r="E5" s="1"/>
-      <x:c r="F5" s="1"/>
-      <x:c r="G5" s="1"/>
+      <x:c r="B2" s="16"/>
+      <x:c r="C2" s="16"/>
+      <x:c r="D2" s="16"/>
+      <x:c r="E2" s="16"/>
+      <x:c r="F2" s="16"/>
+      <x:c r="G2" s="16"/>
+    </x:row>
+    <x:row r="3" ht="8" customHeight="1">
+      <x:c r="A3" s="18"/>
+      <x:c r="B3" s="18"/>
+      <x:c r="C3" s="18"/>
+      <x:c r="D3" s="18"/>
+      <x:c r="E3" s="18"/>
+      <x:c r="F3" s="18"/>
+      <x:c r="G3" s="18"/>
+    </x:row>
+    <x:row r="4" ht="20" customHeight="1">
+      <x:c r="A4" s="18" t="str">
+        <x:v>Source: 空白範本（未提供量測結果）</x:v>
+      </x:c>
+      <x:c r="B4" s="18"/>
+      <x:c r="C4" s="18"/>
+      <x:c r="D4" s="18"/>
+      <x:c r="E4" s="18"/>
+      <x:c r="F4" s="18"/>
+      <x:c r="G4" s="18"/>
+    </x:row>
+    <x:row r="5" ht="20" customHeight="1">
+      <x:c r="A5" s="18" t="str">
+        <x:v>SU / MU (Mbps)</x:v>
+      </x:c>
+      <x:c r="B5" s="18"/>
+      <x:c r="C5" s="18"/>
+      <x:c r="D5" s="18"/>
+      <x:c r="E5" s="18"/>
+      <x:c r="F5" s="18"/>
+      <x:c r="G5" s="18"/>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="8" t="str">
+      <x:c r="A6" s="36" t="str">
         <x:v>Band/Config</x:v>
       </x:c>
-      <x:c r="B6" s="8" t="str">
+      <x:c r="B6" s="36" t="str">
         <x:v>Channel</x:v>
       </x:c>
-      <x:c r="C6" s="8" t="str">
+      <x:c r="C6" s="36" t="str">
         <x:v>Direction</x:v>
       </x:c>
-      <x:c r="D6" s="8" t="str">
+      <x:c r="D6" s="36" t="str">
         <x:v>Gain Criteria</x:v>
       </x:c>
-      <x:c r="E6" s="8" t="str">
+      <x:c r="E6" s="36" t="str">
         <x:v>SU</x:v>
       </x:c>
-      <x:c r="F6" s="8" t="str">
+      <x:c r="F6" s="36" t="str">
         <x:v>MU</x:v>
       </x:c>
-      <x:c r="G6" s="8" t="str">
+      <x:c r="G6" s="36" t="str">
         <x:v>Gain</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="9" t="str">
+      <x:c r="A7" s="28" t="str">
         <x:v>6G_UHR320</x:v>
       </x:c>
-      <x:c r="B7" s="11" t="n">
+      <x:c r="B7" s="39" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="C7" s="9" t="str">
+      <x:c r="C7" s="28" t="str">
         <x:v>UL</x:v>
       </x:c>
-      <x:c r="D7" s="10"/>
-      <x:c r="E7" s="13"/>
-      <x:c r="F7" s="13"/>
-      <x:c r="G7" s="14"/>
+      <x:c r="D7" s="28"/>
+      <x:c r="E7" s="37"/>
+      <x:c r="F7" s="37"/>
+      <x:c r="G7" s="37"/>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="9" t="str">
+      <x:c r="A8" s="32" t="str">
         <x:v>6G_UHR320</x:v>
       </x:c>
-      <x:c r="B8" s="11" t="n">
+      <x:c r="B8" s="40" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="C8" s="9" t="str">
+      <x:c r="C8" s="32" t="str">
         <x:v>DL</x:v>
       </x:c>
-      <x:c r="D8" s="10"/>
-      <x:c r="E8" s="13"/>
-      <x:c r="F8" s="13"/>
-      <x:c r="G8" s="14"/>
+      <x:c r="D8" s="32"/>
+      <x:c r="E8" s="38"/>
+      <x:c r="F8" s="38"/>
+      <x:c r="G8" s="38"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="1"/>
@@ -644,9 +755,20 @@
       <x:c r="G30" s="1"/>
     </x:row>
   </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A3:G3"/>
+    <x:mergeCell ref="A4:G4"/>
+    <x:mergeCell ref="A5:G5"/>
+  </x:mergeCells>
+  <x:printOptions horizontalCentered="1" gridLines="0"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
+  <x:pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <x:headerFooter>
+    <x:oddFooter>&amp;R&amp;P / &amp;N</x:oddFooter>
+  </x:headerFooter>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R818780c50b06401e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redeca699dc5340e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>